<commit_message>
Uday member changes (pages/excel/core) - base 9f99b6c
</commit_message>
<xml_diff>
--- a/lorenzo-playwright-kdf/excelFramework/testcases/HealthIssues/LSTP_HealthIssues_WF001.xlsx
+++ b/lorenzo-playwright-kdf/excelFramework/testcases/HealthIssues/LSTP_HealthIssues_WF001.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mkashetti\ORBIS PAS UKI-LZO\ORBIS PAS UKI-LZO\ORBIS PAS UKI-LZO\lorenzo-playwright-kdf\excelFramework\testcases\HealthIssues\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6960D47-BE93-4940-BF6D-6A77E1D76B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D17CB618-9196-482B-9C2B-6E642154D2C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E23F6686-B9F0-4F90-BA49-870832A24F22}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E23F6686-B9F0-4F90-BA49-870832A24F22}"/>
   </bookViews>
   <sheets>
     <sheet name="TestExecution" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="900" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="425">
   <si>
     <t>StepNo</t>
   </si>
@@ -1152,6 +1152,9 @@
     <t>tbl_Alertname</t>
   </si>
   <si>
+    <t>Verify the recorded alert</t>
+  </si>
+  <si>
     <t>txt_Alertname</t>
   </si>
   <si>
@@ -1324,15 +1327,6 @@
   </si>
   <si>
     <t>pageReopenalert</t>
-  </si>
-  <si>
-    <t>Verify the recorded alert name</t>
-  </si>
-  <si>
-    <t>Verify the recorded alert tyoe</t>
-  </si>
-  <si>
-    <t>ALERT_INFO_SOURCE_MODIFY</t>
   </si>
 </sst>
 </file>
@@ -1960,24 +1954,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDF7DBF7-1927-46F1-B009-E048600E0640}">
   <dimension ref="A1:K182"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.6328125" style="7" customWidth="1"/>
-    <col min="2" max="2" width="66.54296875" style="7" customWidth="1"/>
-    <col min="3" max="3" width="27.6328125" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.7109375" style="7" customWidth="1"/>
+    <col min="2" max="2" width="66.5703125" style="7" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" style="7" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" style="7" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="25" style="7" customWidth="1"/>
-    <col min="7" max="7" width="8.6328125" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" style="7" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.54296875" style="7" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="27.54296875" style="7" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="27.36328125" style="7" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="41.54296875" style="7" customWidth="1"/>
-    <col min="13" max="16384" width="8.6328125" style="7"/>
+    <col min="9" max="9" width="19.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="27.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="27.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="41.5703125" style="7" customWidth="1"/>
+    <col min="13" max="16384" width="8.7109375" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -2012,7 +2006,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -2037,7 +2031,7 @@
       </c>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <v>2</v>
       </c>
@@ -2062,7 +2056,7 @@
       </c>
       <c r="K3" s="8"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
         <v>3</v>
       </c>
@@ -2085,7 +2079,7 @@
       <c r="J4" s="8"/>
       <c r="K4" s="8"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="8">
         <v>4</v>
       </c>
@@ -2108,7 +2102,7 @@
       <c r="J5" s="8"/>
       <c r="K5" s="8"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="8">
         <v>5</v>
       </c>
@@ -2133,7 +2127,7 @@
       <c r="J6" s="8"/>
       <c r="K6" s="8"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="8">
         <v>6</v>
       </c>
@@ -2156,7 +2150,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="8"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="8">
         <v>7</v>
       </c>
@@ -2181,7 +2175,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="8"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
         <v>8</v>
       </c>
@@ -2204,7 +2198,7 @@
       <c r="J9" s="8"/>
       <c r="K9" s="8"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="8">
         <v>9</v>
       </c>
@@ -2227,7 +2221,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="8"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
         <v>10</v>
       </c>
@@ -2252,7 +2246,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="8"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="8">
         <v>11</v>
       </c>
@@ -2287,7 +2281,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="8">
         <v>12</v>
       </c>
@@ -2310,7 +2304,7 @@
       </c>
       <c r="K13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8">
         <v>13</v>
       </c>
@@ -2333,7 +2327,7 @@
       </c>
       <c r="K14" s="8"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="8">
         <v>14</v>
       </c>
@@ -2358,7 +2352,7 @@
       </c>
       <c r="K15" s="8"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="8">
         <v>15</v>
       </c>
@@ -2383,7 +2377,7 @@
       </c>
       <c r="K16" s="8"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="8">
         <v>16</v>
       </c>
@@ -2408,7 +2402,7 @@
       </c>
       <c r="K17" s="8"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="8">
         <v>17</v>
       </c>
@@ -2431,7 +2425,7 @@
       <c r="J18" s="8"/>
       <c r="K18" s="8"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="8">
         <v>18</v>
       </c>
@@ -2456,7 +2450,7 @@
       </c>
       <c r="K19" s="8"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="8">
         <v>19</v>
       </c>
@@ -2479,7 +2473,7 @@
       <c r="J20" s="8"/>
       <c r="K20" s="8"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="8">
         <v>20</v>
       </c>
@@ -2502,7 +2496,7 @@
       <c r="J21" s="8"/>
       <c r="K21" s="8"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="8">
         <v>21</v>
       </c>
@@ -2527,7 +2521,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="8">
         <v>22</v>
       </c>
@@ -2552,7 +2546,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="8">
         <v>23</v>
       </c>
@@ -2575,7 +2569,7 @@
       <c r="J24" s="8"/>
       <c r="K24" s="8"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="8">
         <v>24</v>
       </c>
@@ -2598,7 +2592,7 @@
       </c>
       <c r="K25" s="8"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="8">
         <v>25</v>
       </c>
@@ -2621,7 +2615,7 @@
       <c r="J26" s="8"/>
       <c r="K26" s="8"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="8">
         <v>26</v>
       </c>
@@ -2644,7 +2638,7 @@
       </c>
       <c r="K27" s="8"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="8">
         <v>27</v>
       </c>
@@ -2667,7 +2661,7 @@
       </c>
       <c r="K28" s="8"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="8">
         <v>28</v>
       </c>
@@ -2690,7 +2684,7 @@
       </c>
       <c r="K29" s="8"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="8">
         <v>29</v>
       </c>
@@ -2715,7 +2709,7 @@
       </c>
       <c r="K30" s="8"/>
     </row>
-    <row r="31" spans="1:11" ht="16.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8">
         <v>30</v>
       </c>
@@ -2738,7 +2732,7 @@
       </c>
       <c r="K31" s="8"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="8">
         <v>31</v>
       </c>
@@ -2763,7 +2757,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="8">
         <v>32</v>
       </c>
@@ -2788,7 +2782,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="8">
         <v>33</v>
       </c>
@@ -2811,7 +2805,7 @@
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="8">
         <v>34</v>
       </c>
@@ -2834,7 +2828,7 @@
       </c>
       <c r="K35" s="8"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="8">
         <v>35</v>
       </c>
@@ -2857,7 +2851,7 @@
       <c r="J36" s="8"/>
       <c r="K36" s="8"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="8">
         <v>36</v>
       </c>
@@ -2880,7 +2874,7 @@
       <c r="J37" s="8"/>
       <c r="K37" s="8"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="8">
         <v>37</v>
       </c>
@@ -2903,7 +2897,7 @@
       </c>
       <c r="K38" s="8"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="8">
         <v>38</v>
       </c>
@@ -2926,7 +2920,7 @@
       <c r="J39" s="8"/>
       <c r="K39" s="8"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="8">
         <v>39</v>
       </c>
@@ -2951,7 +2945,7 @@
       </c>
       <c r="K40" s="8"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="8">
         <v>40</v>
       </c>
@@ -2974,7 +2968,7 @@
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="8">
         <v>41</v>
       </c>
@@ -2997,7 +2991,7 @@
       <c r="J42" s="8"/>
       <c r="K42" s="8"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="8">
         <v>42</v>
       </c>
@@ -3022,7 +3016,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="8">
         <v>43</v>
       </c>
@@ -3045,7 +3039,7 @@
       <c r="J44" s="8"/>
       <c r="K44" s="8"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="8">
         <v>44</v>
       </c>
@@ -3070,7 +3064,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="8">
         <v>45</v>
       </c>
@@ -3095,7 +3089,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="8">
         <v>46</v>
       </c>
@@ -3120,7 +3114,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="8">
         <v>47</v>
       </c>
@@ -3145,7 +3139,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="8">
         <v>48</v>
       </c>
@@ -3166,7 +3160,7 @@
       </c>
       <c r="K49" s="8"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="8">
         <v>49</v>
       </c>
@@ -3191,7 +3185,7 @@
       </c>
       <c r="K50" s="8"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="8">
         <v>50</v>
       </c>
@@ -3216,7 +3210,7 @@
       </c>
       <c r="K51" s="8"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="8">
         <v>51</v>
       </c>
@@ -3241,7 +3235,7 @@
       </c>
       <c r="K52" s="8"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="8">
         <v>52</v>
       </c>
@@ -3264,7 +3258,7 @@
       <c r="J53" s="8"/>
       <c r="K53" s="8"/>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="8">
         <v>53</v>
       </c>
@@ -3289,7 +3283,7 @@
       </c>
       <c r="K54" s="8"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="8">
         <v>54</v>
       </c>
@@ -3312,7 +3306,7 @@
       <c r="J55" s="8"/>
       <c r="K55" s="8"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="8">
         <v>55</v>
       </c>
@@ -3335,7 +3329,7 @@
       <c r="J56" s="8"/>
       <c r="K56" s="8"/>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="8">
         <v>56</v>
       </c>
@@ -3358,7 +3352,7 @@
       <c r="J57" s="8"/>
       <c r="K57" s="8"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="8">
         <v>57</v>
       </c>
@@ -3381,7 +3375,7 @@
       </c>
       <c r="K58" s="8"/>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="8">
         <v>58</v>
       </c>
@@ -3402,7 +3396,7 @@
       </c>
       <c r="K59" s="8"/>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="8">
         <v>59</v>
       </c>
@@ -3427,7 +3421,7 @@
       </c>
       <c r="K60" s="8"/>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="8">
         <v>60</v>
       </c>
@@ -3450,7 +3444,7 @@
       </c>
       <c r="K61" s="8"/>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="8">
         <v>61</v>
       </c>
@@ -3473,7 +3467,7 @@
       <c r="J62" s="8"/>
       <c r="K62" s="8"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="8">
         <v>62</v>
       </c>
@@ -3494,7 +3488,7 @@
       <c r="J63" s="8"/>
       <c r="K63" s="8"/>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="8">
         <v>63</v>
       </c>
@@ -3517,7 +3511,7 @@
       <c r="J64" s="12"/>
       <c r="K64" s="8"/>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="8">
         <v>64</v>
       </c>
@@ -3538,7 +3532,7 @@
       <c r="J65" s="8"/>
       <c r="K65" s="8"/>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="8">
         <v>65</v>
       </c>
@@ -3561,7 +3555,7 @@
       <c r="J66" s="8"/>
       <c r="K66" s="8"/>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="8">
         <v>66</v>
       </c>
@@ -3582,7 +3576,7 @@
       </c>
       <c r="K67" s="8"/>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="8">
         <v>67</v>
       </c>
@@ -3609,7 +3603,7 @@
       </c>
       <c r="K68" s="8"/>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="8">
         <v>68</v>
       </c>
@@ -3630,7 +3624,7 @@
       <c r="J69" s="8"/>
       <c r="K69" s="8"/>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="8">
         <v>69</v>
       </c>
@@ -3653,7 +3647,7 @@
       <c r="J70" s="12"/>
       <c r="K70" s="8"/>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="8">
         <v>70</v>
       </c>
@@ -3676,7 +3670,7 @@
       <c r="J71" s="12"/>
       <c r="K71" s="8"/>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="8">
         <v>71</v>
       </c>
@@ -3699,7 +3693,7 @@
       </c>
       <c r="K72" s="8"/>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="8">
         <v>72</v>
       </c>
@@ -3728,7 +3722,7 @@
       </c>
       <c r="K73" s="8"/>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="8">
         <v>73</v>
       </c>
@@ -3753,7 +3747,7 @@
       <c r="J74" s="12"/>
       <c r="K74" s="8"/>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="8">
         <v>74</v>
       </c>
@@ -3776,7 +3770,7 @@
       <c r="J75" s="12"/>
       <c r="K75" s="8"/>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="8">
         <v>75</v>
       </c>
@@ -3799,7 +3793,7 @@
       </c>
       <c r="K76" s="8"/>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="8">
         <v>76</v>
       </c>
@@ -3822,7 +3816,7 @@
       <c r="J77" s="12"/>
       <c r="K77" s="8"/>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="8">
         <v>77</v>
       </c>
@@ -3845,7 +3839,7 @@
       </c>
       <c r="K78" s="8"/>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="8">
         <v>78</v>
       </c>
@@ -3868,7 +3862,7 @@
       </c>
       <c r="K79" s="8"/>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="8">
         <v>79</v>
       </c>
@@ -3891,7 +3885,7 @@
       <c r="J80" s="8"/>
       <c r="K80" s="8"/>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="8">
         <v>80</v>
       </c>
@@ -3912,7 +3906,7 @@
       <c r="J81" s="8"/>
       <c r="K81" s="8"/>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="8">
         <v>81</v>
       </c>
@@ -3935,7 +3929,7 @@
       <c r="J82" s="8"/>
       <c r="K82" s="8"/>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="8">
         <v>82</v>
       </c>
@@ -3956,7 +3950,7 @@
       <c r="J83" s="8"/>
       <c r="K83" s="8"/>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="8">
         <v>83</v>
       </c>
@@ -3976,12 +3970,14 @@
       <c r="G84" s="8"/>
       <c r="H84" s="8"/>
       <c r="I84" s="8"/>
-      <c r="J84" s="8"/>
+      <c r="J84" s="8" t="s">
+        <v>396</v>
+      </c>
       <c r="K84" s="8" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" s="8">
         <v>84</v>
       </c>
@@ -3996,17 +3992,19 @@
       </c>
       <c r="E85" s="8"/>
       <c r="F85" s="8" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="G85" s="8"/>
       <c r="H85" s="8"/>
       <c r="I85" s="8"/>
-      <c r="J85" s="8"/>
+      <c r="J85" s="8" t="s">
+        <v>391</v>
+      </c>
       <c r="K85" s="8" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="8">
         <v>85</v>
       </c>
@@ -4026,12 +4024,14 @@
       <c r="G86" s="8"/>
       <c r="H86" s="8"/>
       <c r="I86" s="8"/>
-      <c r="J86" s="8"/>
+      <c r="J86" s="8" t="s">
+        <v>214</v>
+      </c>
       <c r="K86" s="8" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" s="8">
         <v>86</v>
       </c>
@@ -4054,7 +4054,7 @@
       <c r="J87" s="8"/>
       <c r="K87" s="8"/>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" s="8">
         <v>87</v>
       </c>
@@ -4077,7 +4077,7 @@
       <c r="J88" s="8"/>
       <c r="K88" s="8"/>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" s="8">
         <v>88</v>
       </c>
@@ -4098,18 +4098,18 @@
       <c r="J89" s="8"/>
       <c r="K89" s="8"/>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" s="8">
         <v>89</v>
       </c>
       <c r="B90" s="8" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C90" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D90" s="16" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E90" s="8"/>
       <c r="F90" s="8" t="s">
@@ -4122,23 +4122,25 @@
         <v>113</v>
       </c>
       <c r="I90" s="8"/>
-      <c r="J90" s="8"/>
+      <c r="J90" s="8" t="s">
+        <v>391</v>
+      </c>
       <c r="K90" s="8" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" s="8">
         <v>90</v>
       </c>
       <c r="B91" s="8" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C91" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D91" s="16" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E91" s="8"/>
       <c r="F91" s="8" t="s">
@@ -4151,23 +4153,25 @@
         <v>113</v>
       </c>
       <c r="I91" s="8"/>
-      <c r="J91" s="8"/>
+      <c r="J91" s="8" t="s">
+        <v>396</v>
+      </c>
       <c r="K91" s="8" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" s="8">
         <v>91</v>
       </c>
       <c r="B92" s="8" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C92" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D92" s="16" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E92" s="8"/>
       <c r="F92" s="8" t="s">
@@ -4180,12 +4184,14 @@
         <v>113</v>
       </c>
       <c r="I92" s="8"/>
-      <c r="J92" s="8"/>
+      <c r="J92" s="8" t="s">
+        <v>214</v>
+      </c>
       <c r="K92" s="8" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" s="8">
         <v>92</v>
       </c>
@@ -4206,7 +4212,7 @@
       </c>
       <c r="K93" s="8"/>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" s="8">
         <v>93</v>
       </c>
@@ -4227,7 +4233,7 @@
       <c r="J94" s="8"/>
       <c r="K94" s="8"/>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95" s="8">
         <v>94</v>
       </c>
@@ -4250,7 +4256,7 @@
       <c r="J95" s="8"/>
       <c r="K95" s="8"/>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96" s="8">
         <v>95</v>
       </c>
@@ -4258,7 +4264,7 @@
         <v>174</v>
       </c>
       <c r="C96" s="8" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D96" s="8"/>
       <c r="E96" s="8"/>
@@ -4271,7 +4277,7 @@
       <c r="J96" s="8"/>
       <c r="K96" s="8"/>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A97" s="8">
         <v>96</v>
       </c>
@@ -4279,7 +4285,7 @@
         <v>175</v>
       </c>
       <c r="C97" s="8" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D97" s="8" t="s">
         <v>176</v>
@@ -4292,11 +4298,11 @@
       <c r="H97" s="8"/>
       <c r="I97" s="8"/>
       <c r="J97" s="8" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="K97" s="8"/>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A98" s="8">
         <v>97</v>
       </c>
@@ -4304,7 +4310,7 @@
         <v>178</v>
       </c>
       <c r="C98" s="8" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D98" s="8" t="s">
         <v>81</v>
@@ -4319,7 +4325,7 @@
       <c r="J98" s="8"/>
       <c r="K98" s="8"/>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A99" s="8">
         <v>98</v>
       </c>
@@ -4340,12 +4346,12 @@
       <c r="J99" s="8"/>
       <c r="K99" s="8"/>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A100" s="8">
         <v>99</v>
       </c>
       <c r="B100" s="8" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C100" s="8" t="s">
         <v>18</v>
@@ -4353,17 +4359,17 @@
       <c r="D100" s="8"/>
       <c r="E100" s="8"/>
       <c r="F100" s="8" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="G100" s="8"/>
       <c r="H100" s="8"/>
       <c r="I100" s="8"/>
       <c r="J100" s="8" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K100" s="8"/>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A101" s="8">
         <v>100</v>
       </c>
@@ -4374,7 +4380,7 @@
         <v>18</v>
       </c>
       <c r="D101" s="8" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="E101" s="8"/>
       <c r="F101" s="8" t="s">
@@ -4388,11 +4394,11 @@
       </c>
       <c r="I101" s="8"/>
       <c r="J101" s="8" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="K101" s="8"/>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A102" s="8">
         <v>101</v>
       </c>
@@ -4413,7 +4419,7 @@
       </c>
       <c r="K102" s="8"/>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A103" s="8">
         <v>102</v>
       </c>
@@ -4436,7 +4442,7 @@
       <c r="J103" s="8"/>
       <c r="K103" s="8"/>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A104" s="8">
         <v>103</v>
       </c>
@@ -4444,7 +4450,7 @@
         <v>184</v>
       </c>
       <c r="C104" s="8" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D104" s="8"/>
       <c r="E104" s="8"/>
@@ -4457,18 +4463,18 @@
       <c r="J104" s="8"/>
       <c r="K104" s="8"/>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A105" s="8">
         <v>104</v>
       </c>
       <c r="B105" s="8" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C105" s="8" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D105" s="8" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E105" s="8"/>
       <c r="F105" s="8" t="s">
@@ -4486,7 +4492,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A106" s="8">
         <v>105</v>
       </c>
@@ -4494,7 +4500,7 @@
         <v>185</v>
       </c>
       <c r="C106" s="8" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D106" s="8" t="s">
         <v>120</v>
@@ -4506,12 +4512,14 @@
       <c r="G106" s="8"/>
       <c r="H106" s="8"/>
       <c r="I106" s="8"/>
-      <c r="J106" s="8"/>
+      <c r="J106" s="8" t="s">
+        <v>400</v>
+      </c>
       <c r="K106" s="8" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A107" s="8">
         <v>106</v>
       </c>
@@ -4519,7 +4527,7 @@
         <v>187</v>
       </c>
       <c r="C107" s="8" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D107" s="8" t="s">
         <v>91</v>
@@ -4534,7 +4542,7 @@
       <c r="J107" s="8"/>
       <c r="K107" s="8"/>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A108" s="8">
         <v>107</v>
       </c>
@@ -4542,7 +4550,7 @@
         <v>188</v>
       </c>
       <c r="C108" s="8" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D108" s="8"/>
       <c r="E108" s="8"/>
@@ -4555,7 +4563,7 @@
       <c r="J108" s="8"/>
       <c r="K108" s="8"/>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A109" s="8">
         <v>108</v>
       </c>
@@ -4578,18 +4586,18 @@
       <c r="J109" s="8"/>
       <c r="K109" s="8"/>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A110" s="8">
         <v>109</v>
       </c>
       <c r="B110" s="8" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C110" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D110" s="16" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E110" s="8"/>
       <c r="F110" s="8" t="s">
@@ -4602,23 +4610,25 @@
         <v>113</v>
       </c>
       <c r="I110" s="8"/>
-      <c r="J110" s="8"/>
+      <c r="J110" s="8" t="s">
+        <v>391</v>
+      </c>
       <c r="K110" s="8" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A111" s="8">
         <v>110</v>
       </c>
       <c r="B111" s="8" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C111" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D111" s="16" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E111" s="8"/>
       <c r="F111" s="8" t="s">
@@ -4632,11 +4642,11 @@
       </c>
       <c r="I111" s="8"/>
       <c r="J111" s="8" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="K111" s="8"/>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A112" s="8">
         <v>111</v>
       </c>
@@ -4657,7 +4667,7 @@
       </c>
       <c r="K112" s="8"/>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113" s="8">
         <v>112</v>
       </c>
@@ -4678,7 +4688,7 @@
       <c r="J113" s="8"/>
       <c r="K113" s="8"/>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114" s="8">
         <v>113</v>
       </c>
@@ -4701,7 +4711,7 @@
       <c r="J114" s="8"/>
       <c r="K114" s="8"/>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" s="8">
         <v>114</v>
       </c>
@@ -4709,7 +4719,7 @@
         <v>193</v>
       </c>
       <c r="C115" s="8" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D115" s="8"/>
       <c r="E115" s="8"/>
@@ -4722,18 +4732,18 @@
       <c r="J115" s="8"/>
       <c r="K115" s="8"/>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" s="8">
         <v>115</v>
       </c>
       <c r="B116" s="8" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C116" s="8" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D116" s="8" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E116" s="8"/>
       <c r="F116" s="8" t="s">
@@ -4751,7 +4761,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" s="8">
         <v>116</v>
       </c>
@@ -4759,7 +4769,7 @@
         <v>194</v>
       </c>
       <c r="C117" s="8" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D117" s="8" t="s">
         <v>195</v>
@@ -4771,12 +4781,14 @@
       <c r="G117" s="8"/>
       <c r="H117" s="8"/>
       <c r="I117" s="8"/>
-      <c r="J117" s="8"/>
+      <c r="J117" s="8" t="s">
+        <v>408</v>
+      </c>
       <c r="K117" s="8" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" s="8">
         <v>117</v>
       </c>
@@ -4784,7 +4796,7 @@
         <v>197</v>
       </c>
       <c r="C118" s="8" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D118" s="8" t="s">
         <v>91</v>
@@ -4799,7 +4811,7 @@
       <c r="J118" s="8"/>
       <c r="K118" s="8"/>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" s="8">
         <v>118</v>
       </c>
@@ -4807,7 +4819,7 @@
         <v>198</v>
       </c>
       <c r="C119" s="8" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D119" s="8"/>
       <c r="E119" s="8"/>
@@ -4820,18 +4832,18 @@
       <c r="J119" s="8"/>
       <c r="K119" s="8"/>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" s="8">
         <v>119</v>
       </c>
       <c r="B120" s="8" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C120" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D120" s="16" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E120" s="8"/>
       <c r="F120" s="8" t="s">
@@ -4844,23 +4856,25 @@
         <v>113</v>
       </c>
       <c r="I120" s="8"/>
-      <c r="J120" s="8"/>
+      <c r="J120" s="8" t="s">
+        <v>391</v>
+      </c>
       <c r="K120" s="8" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" s="8">
         <v>120</v>
       </c>
       <c r="B121" s="8" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C121" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D121" s="16" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E121" s="8"/>
       <c r="F121" s="8" t="s">
@@ -4874,11 +4888,11 @@
       </c>
       <c r="I121" s="8"/>
       <c r="J121" s="8" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K121" s="8"/>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" s="8">
         <v>121</v>
       </c>
@@ -4899,7 +4913,7 @@
       </c>
       <c r="K122" s="8"/>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" s="8">
         <v>122</v>
       </c>
@@ -4922,7 +4936,7 @@
       <c r="J123" s="8"/>
       <c r="K123" s="8"/>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124" s="8">
         <v>123</v>
       </c>
@@ -4930,7 +4944,7 @@
         <v>202</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D124" s="8"/>
       <c r="E124" s="8"/>
@@ -4943,18 +4957,18 @@
       <c r="J124" s="8"/>
       <c r="K124" s="8"/>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125" s="8">
         <v>124</v>
       </c>
       <c r="B125" s="8" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C125" s="8" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D125" s="8" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E125" s="8"/>
       <c r="F125" s="8" t="s">
@@ -4972,7 +4986,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126" s="8">
         <v>125</v>
       </c>
@@ -4980,7 +4994,7 @@
         <v>203</v>
       </c>
       <c r="C126" s="8" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D126" s="8" t="s">
         <v>140</v>
@@ -4992,12 +5006,14 @@
       <c r="G126" s="8"/>
       <c r="H126" s="8"/>
       <c r="I126" s="8"/>
-      <c r="J126" s="8"/>
+      <c r="J126" s="8" t="s">
+        <v>409</v>
+      </c>
       <c r="K126" s="8" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127" s="8">
         <v>126</v>
       </c>
@@ -5005,7 +5021,7 @@
         <v>205</v>
       </c>
       <c r="C127" s="8" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D127" s="8" t="s">
         <v>143</v>
@@ -5020,7 +5036,7 @@
       <c r="J127" s="8"/>
       <c r="K127" s="8"/>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128" s="8">
         <v>127</v>
       </c>
@@ -5028,7 +5044,7 @@
         <v>206</v>
       </c>
       <c r="C128" s="8" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D128" s="8" t="s">
         <v>91</v>
@@ -5043,7 +5059,7 @@
       <c r="J128" s="8"/>
       <c r="K128" s="8"/>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A129" s="8">
         <v>128</v>
       </c>
@@ -5064,7 +5080,7 @@
       <c r="J129" s="8"/>
       <c r="K129" s="8"/>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A130" s="8">
         <v>129</v>
       </c>
@@ -5087,18 +5103,18 @@
       <c r="J130" s="8"/>
       <c r="K130" s="8"/>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A131" s="8">
         <v>130</v>
       </c>
       <c r="B131" s="8" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C131" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D131" s="16" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E131" s="8"/>
       <c r="F131" s="8" t="s">
@@ -5111,23 +5127,25 @@
         <v>113</v>
       </c>
       <c r="I131" s="8"/>
-      <c r="J131" s="8"/>
+      <c r="J131" s="8" t="s">
+        <v>391</v>
+      </c>
       <c r="K131" s="8" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A132" s="8">
         <v>131</v>
       </c>
       <c r="B132" s="8" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C132" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D132" s="16" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E132" s="8"/>
       <c r="F132" s="8" t="s">
@@ -5141,16 +5159,16 @@
       </c>
       <c r="I132" s="8"/>
       <c r="J132" s="8" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K132" s="8"/>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A133" s="8">
         <v>132</v>
       </c>
       <c r="B133" s="12" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C133" s="8" t="s">
         <v>18</v>
@@ -5166,7 +5184,7 @@
       <c r="J133" s="12"/>
       <c r="K133" s="8"/>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A134" s="8">
         <v>133</v>
       </c>
@@ -5189,7 +5207,7 @@
       <c r="J134" s="12"/>
       <c r="K134" s="8"/>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A135" s="8">
         <v>134</v>
       </c>
@@ -5212,7 +5230,7 @@
       </c>
       <c r="K135" s="8"/>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A136" s="8">
         <v>135</v>
       </c>
@@ -5235,7 +5253,7 @@
       <c r="J136" s="12"/>
       <c r="K136" s="8"/>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A137" s="8">
         <v>136</v>
       </c>
@@ -5243,7 +5261,7 @@
         <v>104</v>
       </c>
       <c r="C137" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D137" s="8" t="s">
         <v>105</v>
@@ -5255,12 +5273,14 @@
       <c r="G137" s="8"/>
       <c r="H137" s="8"/>
       <c r="I137" s="8"/>
-      <c r="J137" s="8"/>
+      <c r="J137" s="8" t="s">
+        <v>354</v>
+      </c>
       <c r="K137" s="8" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A138" s="8">
         <v>137</v>
       </c>
@@ -5268,7 +5288,7 @@
         <v>278</v>
       </c>
       <c r="C138" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D138" s="8"/>
       <c r="E138" s="8"/>
@@ -5283,7 +5303,7 @@
       </c>
       <c r="K138" s="8"/>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A139" s="8">
         <v>138</v>
       </c>
@@ -5291,7 +5311,7 @@
         <v>364</v>
       </c>
       <c r="C139" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D139" s="8" t="s">
         <v>108</v>
@@ -5306,7 +5326,7 @@
       <c r="J139" s="8"/>
       <c r="K139" s="8"/>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A140" s="8">
         <v>139</v>
       </c>
@@ -5314,7 +5334,7 @@
         <v>107</v>
       </c>
       <c r="C140" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D140" s="8" t="s">
         <v>365</v>
@@ -5333,7 +5353,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A141" s="8">
         <v>140</v>
       </c>
@@ -5341,7 +5361,7 @@
         <v>110</v>
       </c>
       <c r="C141" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D141" s="8" t="s">
         <v>111</v>
@@ -5353,12 +5373,14 @@
       <c r="G141" s="8"/>
       <c r="H141" s="8"/>
       <c r="I141" s="8"/>
-      <c r="J141" s="8"/>
+      <c r="J141" s="8" t="s">
+        <v>363</v>
+      </c>
       <c r="K141" s="8" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A142" s="8">
         <v>141</v>
       </c>
@@ -5366,7 +5388,7 @@
         <v>112</v>
       </c>
       <c r="C142" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D142" s="8" t="s">
         <v>81</v>
@@ -5381,7 +5403,7 @@
       <c r="J142" s="8"/>
       <c r="K142" s="8"/>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A143" s="8">
         <v>142</v>
       </c>
@@ -5400,18 +5422,18 @@
       <c r="J143" s="8"/>
       <c r="K143" s="8"/>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A144" s="8">
         <v>143</v>
       </c>
       <c r="B144" s="8" t="s">
-        <v>425</v>
+        <v>366</v>
       </c>
       <c r="C144" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D144" s="16" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E144" s="8"/>
       <c r="F144" s="8" t="s">
@@ -5429,18 +5451,18 @@
         <v>106</v>
       </c>
     </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A145" s="8">
         <v>144</v>
       </c>
       <c r="B145" s="8" t="s">
-        <v>424</v>
+        <v>366</v>
       </c>
       <c r="C145" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D145" s="16" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E145" s="8"/>
       <c r="F145" s="8" t="s">
@@ -5458,12 +5480,12 @@
         <v>109</v>
       </c>
     </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A146" s="8">
         <v>145</v>
       </c>
       <c r="B146" s="8" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C146" s="16"/>
       <c r="D146" s="16"/>
@@ -5479,7 +5501,7 @@
       </c>
       <c r="K146" s="8"/>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A147" s="8">
         <v>146</v>
       </c>
@@ -5502,7 +5524,7 @@
       <c r="J147" s="8"/>
       <c r="K147" s="8"/>
     </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A148" s="8">
         <v>147</v>
       </c>
@@ -5521,15 +5543,15 @@
       <c r="J148" s="8"/>
       <c r="K148" s="8"/>
     </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A149" s="8">
         <v>148</v>
       </c>
       <c r="B149" s="8" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C149" s="8" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D149" s="8" t="s">
         <v>164</v>
@@ -5541,20 +5563,22 @@
       <c r="G149" s="8"/>
       <c r="H149" s="8"/>
       <c r="I149" s="8"/>
-      <c r="J149" s="8"/>
+      <c r="J149" s="8" t="s">
+        <v>356</v>
+      </c>
       <c r="K149" s="8" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.35">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A150" s="8">
         <v>149</v>
       </c>
       <c r="B150" s="8" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C150" s="8" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D150" s="8" t="s">
         <v>81</v>
@@ -5569,7 +5593,7 @@
       <c r="J150" s="8"/>
       <c r="K150" s="8"/>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A151" s="8">
         <v>150</v>
       </c>
@@ -5588,18 +5612,18 @@
       <c r="J151" s="8"/>
       <c r="K151" s="8"/>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A152" s="8">
         <v>151</v>
       </c>
       <c r="B152" s="8" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C152" s="16" t="s">
         <v>18</v>
       </c>
       <c r="D152" s="16" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E152" s="8"/>
       <c r="F152" s="8" t="s">
@@ -5614,15 +5638,15 @@
       <c r="I152" s="8"/>
       <c r="J152" s="8"/>
       <c r="K152" s="8" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.35">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A153" s="8">
         <v>152</v>
       </c>
       <c r="B153" s="8" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C153" s="16"/>
       <c r="D153" s="16"/>
@@ -5638,12 +5662,12 @@
       </c>
       <c r="K153" s="8"/>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A154" s="8">
         <v>153</v>
       </c>
       <c r="B154" s="8" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C154" s="8" t="s">
         <v>18</v>
@@ -5661,18 +5685,18 @@
       <c r="J154" s="8"/>
       <c r="K154" s="8"/>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A155" s="8">
         <v>154</v>
       </c>
       <c r="B155" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C155" s="8" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D155" s="16" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E155" s="8"/>
       <c r="F155" s="8" t="s">
@@ -5690,18 +5714,18 @@
         <v>106</v>
       </c>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A156" s="8">
         <v>155</v>
       </c>
       <c r="B156" s="8" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C156" s="8" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D156" s="16" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E156" s="8"/>
       <c r="F156" s="8" t="s">
@@ -5719,15 +5743,15 @@
         <v>109</v>
       </c>
     </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A157" s="8">
         <v>156</v>
       </c>
       <c r="B157" s="8" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C157" s="8" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D157" s="16" t="s">
         <v>120</v>
@@ -5739,20 +5763,22 @@
       <c r="G157" s="8"/>
       <c r="H157" s="8"/>
       <c r="I157" s="8"/>
-      <c r="J157" s="8"/>
+      <c r="J157" s="8" t="s">
+        <v>357</v>
+      </c>
       <c r="K157" s="8" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A158" s="8">
         <v>157</v>
       </c>
       <c r="B158" s="8" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C158" s="8" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D158" s="8" t="s">
         <v>91</v>
@@ -5767,7 +5793,7 @@
       <c r="J158" s="8"/>
       <c r="K158" s="8"/>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A159" s="8">
         <v>158</v>
       </c>
@@ -5788,7 +5814,7 @@
       <c r="J159" s="8"/>
       <c r="K159" s="8"/>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A160" s="8">
         <v>159</v>
       </c>
@@ -5811,7 +5837,7 @@
       <c r="J160" s="8"/>
       <c r="K160" s="8"/>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A161" s="8">
         <v>160</v>
       </c>
@@ -5834,7 +5860,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A162" s="8">
         <v>161</v>
       </c>
@@ -5845,7 +5871,7 @@
         <v>18</v>
       </c>
       <c r="D162" s="8" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E162" s="8"/>
       <c r="F162" s="8" t="s">
@@ -5859,11 +5885,11 @@
       </c>
       <c r="I162" s="8"/>
       <c r="J162" s="8" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="K162" s="8"/>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A163" s="8">
         <v>162</v>
       </c>
@@ -5884,7 +5910,7 @@
       </c>
       <c r="K163" s="8"/>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A164" s="8">
         <v>163</v>
       </c>
@@ -5907,7 +5933,7 @@
       <c r="J164" s="8"/>
       <c r="K164" s="8"/>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A165" s="8">
         <v>164</v>
       </c>
@@ -5915,7 +5941,7 @@
         <v>128</v>
       </c>
       <c r="C165" s="8" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D165" s="8"/>
       <c r="E165" s="8"/>
@@ -5928,18 +5954,18 @@
       <c r="J165" s="8"/>
       <c r="K165" s="8"/>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A166" s="8">
         <v>165</v>
       </c>
       <c r="B166" s="8" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C166" s="8" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D166" s="16" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E166" s="8"/>
       <c r="F166" s="8" t="s">
@@ -5957,18 +5983,18 @@
         <v>106</v>
       </c>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A167" s="8">
         <v>166</v>
       </c>
       <c r="B167" s="8" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C167" s="8" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D167" s="16" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E167" s="8"/>
       <c r="F167" s="8" t="s">
@@ -5986,7 +6012,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A168" s="8">
         <v>167</v>
       </c>
@@ -5994,7 +6020,7 @@
         <v>129</v>
       </c>
       <c r="C168" s="8" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D168" s="8" t="s">
         <v>130</v>
@@ -6006,12 +6032,14 @@
       <c r="G168" s="8"/>
       <c r="H168" s="8"/>
       <c r="I168" s="8"/>
-      <c r="J168" s="8"/>
+      <c r="J168" s="8" t="s">
+        <v>358</v>
+      </c>
       <c r="K168" s="8" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A169" s="8">
         <v>168</v>
       </c>
@@ -6019,7 +6047,7 @@
         <v>132</v>
       </c>
       <c r="C169" s="8" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D169" s="8" t="s">
         <v>91</v>
@@ -6034,7 +6062,7 @@
       <c r="J169" s="8"/>
       <c r="K169" s="8"/>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A170" s="8">
         <v>169</v>
       </c>
@@ -6055,7 +6083,7 @@
       <c r="J170" s="8"/>
       <c r="K170" s="8"/>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A171" s="8">
         <v>170</v>
       </c>
@@ -6066,7 +6094,7 @@
         <v>18</v>
       </c>
       <c r="D171" s="8" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E171" s="8"/>
       <c r="F171" s="8" t="s">
@@ -6080,11 +6108,11 @@
       </c>
       <c r="I171" s="8"/>
       <c r="J171" s="8" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K171" s="8"/>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A172" s="8">
         <v>171</v>
       </c>
@@ -6105,7 +6133,7 @@
       </c>
       <c r="K172" s="8"/>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A173" s="8">
         <v>172</v>
       </c>
@@ -6128,7 +6156,7 @@
       <c r="J173" s="8"/>
       <c r="K173" s="8"/>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A174" s="8">
         <v>173</v>
       </c>
@@ -6136,7 +6164,7 @@
         <v>138</v>
       </c>
       <c r="C174" s="8" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D174" s="8"/>
       <c r="E174" s="8"/>
@@ -6149,18 +6177,18 @@
       <c r="J174" s="8"/>
       <c r="K174" s="8"/>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A175" s="8">
         <v>174</v>
       </c>
       <c r="B175" s="8" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C175" s="8" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D175" s="16" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E175" s="8"/>
       <c r="F175" s="8" t="s">
@@ -6178,18 +6206,18 @@
         <v>106</v>
       </c>
     </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A176" s="8">
         <v>175</v>
       </c>
       <c r="B176" s="8" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C176" s="8" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D176" s="16" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E176" s="8"/>
       <c r="F176" s="8" t="s">
@@ -6207,7 +6235,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A177" s="8">
         <v>176</v>
       </c>
@@ -6215,7 +6243,7 @@
         <v>139</v>
       </c>
       <c r="C177" s="8" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D177" s="8" t="s">
         <v>140</v>
@@ -6227,12 +6255,14 @@
       <c r="G177" s="8"/>
       <c r="H177" s="8"/>
       <c r="I177" s="8"/>
-      <c r="J177" s="8"/>
+      <c r="J177" s="8" t="s">
+        <v>359</v>
+      </c>
       <c r="K177" s="8" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A178" s="8">
         <v>177</v>
       </c>
@@ -6240,7 +6270,7 @@
         <v>142</v>
       </c>
       <c r="C178" s="8" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D178" s="8" t="s">
         <v>143</v>
@@ -6255,7 +6285,7 @@
       <c r="J178" s="8"/>
       <c r="K178" s="8"/>
     </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A179" s="8">
         <v>178</v>
       </c>
@@ -6263,7 +6293,7 @@
         <v>144</v>
       </c>
       <c r="C179" s="8" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D179" s="8" t="s">
         <v>91</v>
@@ -6278,7 +6308,7 @@
       <c r="J179" s="8"/>
       <c r="K179" s="8"/>
     </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A180" s="8">
         <v>179</v>
       </c>
@@ -6299,7 +6329,7 @@
       <c r="J180" s="8"/>
       <c r="K180" s="8"/>
     </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A181" s="8">
         <v>180</v>
       </c>
@@ -6322,7 +6352,7 @@
       <c r="J181" s="8"/>
       <c r="K181" s="8"/>
     </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A182" s="8">
         <v>181</v>
       </c>
@@ -6333,7 +6363,7 @@
         <v>18</v>
       </c>
       <c r="D182" s="8" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E182" s="8"/>
       <c r="F182" s="8" t="s">
@@ -6347,7 +6377,7 @@
       </c>
       <c r="I182" s="8"/>
       <c r="J182" s="8" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K182" s="8"/>
     </row>
@@ -6372,38 +6402,37 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31674DB1-2F1A-4DBC-BB88-9570360CDD29}">
-  <dimension ref="A1:AB2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AA2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="19.36328125" customWidth="1"/>
-    <col min="12" max="12" width="20.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.6328125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.6328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.6328125" customWidth="1"/>
-    <col min="19" max="19" width="22.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="23.6328125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="26.453125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.54296875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="23.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="22.36328125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="25" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="26.54296875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="19.28515625" customWidth="1"/>
+    <col min="12" max="12" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="25" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="29" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>45</v>
       </c>
@@ -6456,40 +6485,37 @@
         <v>118</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>426</v>
+        <v>121</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="AB1" s="1" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>210</v>
       </c>
@@ -6539,40 +6565,37 @@
         <v>355</v>
       </c>
       <c r="Q2" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
       <c r="R2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="S2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="T2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="U2" t="s">
-        <v>359</v>
+        <v>396</v>
       </c>
       <c r="V2" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="W2" t="s">
+        <v>214</v>
+      </c>
+      <c r="X2" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="X2" t="s">
-        <v>214</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>389</v>
+      <c r="Y2" t="s">
+        <v>400</v>
       </c>
       <c r="Z2" t="s">
-        <v>399</v>
+        <v>408</v>
       </c>
       <c r="AA2" t="s">
-        <v>407</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
   </sheetData>
@@ -6583,13 +6606,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A492E716-2E2C-4117-849D-EDDCA92E50F2}">
   <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.54296875" customWidth="1"/>
+    <col min="1" max="1" width="27.5703125" customWidth="1"/>
     <col min="2" max="2" width="95" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>215</v>
       </c>
@@ -6597,7 +6620,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>217</v>
       </c>
@@ -6605,7 +6628,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>219</v>
       </c>
@@ -6613,7 +6636,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>221</v>
       </c>
@@ -6621,7 +6644,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>223</v>
       </c>
@@ -6629,7 +6652,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>225</v>
       </c>
@@ -6637,7 +6660,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>227</v>
       </c>
@@ -6645,7 +6668,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>229</v>
       </c>
@@ -6653,7 +6676,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>231</v>
       </c>
@@ -6661,7 +6684,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>232</v>
       </c>
@@ -6669,7 +6692,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>233</v>
       </c>
@@ -6677,7 +6700,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>234</v>
       </c>
@@ -6685,7 +6708,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>236</v>
       </c>
@@ -6693,7 +6716,7 @@
         <v>46178</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>237</v>
       </c>
@@ -6701,7 +6724,7 @@
         <v>46178</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>238</v>
       </c>
@@ -6709,7 +6732,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>240</v>
       </c>
@@ -6717,7 +6740,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>242</v>
       </c>
@@ -6725,7 +6748,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>244</v>
       </c>
@@ -6733,7 +6756,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>245</v>
       </c>
@@ -6741,7 +6764,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>247</v>
       </c>
@@ -6757,14 +6780,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E342BCFB-0C06-449E-9D93-F79DC7BEEDFF}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="37" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>249</v>
       </c>
@@ -6775,7 +6798,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>38</v>
       </c>
@@ -6786,7 +6809,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -6797,7 +6820,7 @@
         <v>996289289229</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -6811,10 +6834,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{a4153a30-97aa-49dd-8839-66f72081522c}" enabled="1" method="Standard" siteId="{9ffff5c3-bdfa-4a9d-b595-ff68329945ef}" contentBits="0" removed="0"/>
-</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Sakthi member changes (pages/excel/core) - base 9f99b6c
</commit_message>
<xml_diff>
--- a/lorenzo-playwright-kdf/excelFramework/testcases/HealthIssues/LSTP_HealthIssues_WF001.xlsx
+++ b/lorenzo-playwright-kdf/excelFramework/testcases/HealthIssues/LSTP_HealthIssues_WF001.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mkashetti\ORBIS PAS UKI-LZO\ORBIS PAS UKI-LZO\ORBIS PAS UKI-LZO\lorenzo-playwright-kdf\excelFramework\testcases\HealthIssues\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6960D47-BE93-4940-BF6D-6A77E1D76B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D17CB618-9196-482B-9C2B-6E642154D2C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E23F6686-B9F0-4F90-BA49-870832A24F22}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E23F6686-B9F0-4F90-BA49-870832A24F22}"/>
   </bookViews>
   <sheets>
     <sheet name="TestExecution" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="900" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="425">
   <si>
     <t>StepNo</t>
   </si>
@@ -1152,6 +1152,9 @@
     <t>tbl_Alertname</t>
   </si>
   <si>
+    <t>Verify the recorded alert</t>
+  </si>
+  <si>
     <t>txt_Alertname</t>
   </si>
   <si>
@@ -1324,15 +1327,6 @@
   </si>
   <si>
     <t>pageReopenalert</t>
-  </si>
-  <si>
-    <t>Verify the recorded alert name</t>
-  </si>
-  <si>
-    <t>Verify the recorded alert tyoe</t>
-  </si>
-  <si>
-    <t>ALERT_INFO_SOURCE_MODIFY</t>
   </si>
 </sst>
 </file>
@@ -1960,24 +1954,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDF7DBF7-1927-46F1-B009-E048600E0640}">
   <dimension ref="A1:K182"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.6328125" style="7" customWidth="1"/>
-    <col min="2" max="2" width="66.54296875" style="7" customWidth="1"/>
-    <col min="3" max="3" width="27.6328125" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.7109375" style="7" customWidth="1"/>
+    <col min="2" max="2" width="66.5703125" style="7" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" style="7" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" style="7" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="25" style="7" customWidth="1"/>
-    <col min="7" max="7" width="8.6328125" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" style="7" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.54296875" style="7" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="27.54296875" style="7" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="27.36328125" style="7" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="41.54296875" style="7" customWidth="1"/>
-    <col min="13" max="16384" width="8.6328125" style="7"/>
+    <col min="9" max="9" width="19.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="27.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="27.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="41.5703125" style="7" customWidth="1"/>
+    <col min="13" max="16384" width="8.7109375" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -2012,7 +2006,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -2037,7 +2031,7 @@
       </c>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <v>2</v>
       </c>
@@ -2062,7 +2056,7 @@
       </c>
       <c r="K3" s="8"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
         <v>3</v>
       </c>
@@ -2085,7 +2079,7 @@
       <c r="J4" s="8"/>
       <c r="K4" s="8"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="8">
         <v>4</v>
       </c>
@@ -2108,7 +2102,7 @@
       <c r="J5" s="8"/>
       <c r="K5" s="8"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="8">
         <v>5</v>
       </c>
@@ -2133,7 +2127,7 @@
       <c r="J6" s="8"/>
       <c r="K6" s="8"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="8">
         <v>6</v>
       </c>
@@ -2156,7 +2150,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="8"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="8">
         <v>7</v>
       </c>
@@ -2181,7 +2175,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="8"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
         <v>8</v>
       </c>
@@ -2204,7 +2198,7 @@
       <c r="J9" s="8"/>
       <c r="K9" s="8"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="8">
         <v>9</v>
       </c>
@@ -2227,7 +2221,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="8"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
         <v>10</v>
       </c>
@@ -2252,7 +2246,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="8"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="8">
         <v>11</v>
       </c>
@@ -2287,7 +2281,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="8">
         <v>12</v>
       </c>
@@ -2310,7 +2304,7 @@
       </c>
       <c r="K13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8">
         <v>13</v>
       </c>
@@ -2333,7 +2327,7 @@
       </c>
       <c r="K14" s="8"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="8">
         <v>14</v>
       </c>
@@ -2358,7 +2352,7 @@
       </c>
       <c r="K15" s="8"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="8">
         <v>15</v>
       </c>
@@ -2383,7 +2377,7 @@
       </c>
       <c r="K16" s="8"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="8">
         <v>16</v>
       </c>
@@ -2408,7 +2402,7 @@
       </c>
       <c r="K17" s="8"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="8">
         <v>17</v>
       </c>
@@ -2431,7 +2425,7 @@
       <c r="J18" s="8"/>
       <c r="K18" s="8"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="8">
         <v>18</v>
       </c>
@@ -2456,7 +2450,7 @@
       </c>
       <c r="K19" s="8"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="8">
         <v>19</v>
       </c>
@@ -2479,7 +2473,7 @@
       <c r="J20" s="8"/>
       <c r="K20" s="8"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="8">
         <v>20</v>
       </c>
@@ -2502,7 +2496,7 @@
       <c r="J21" s="8"/>
       <c r="K21" s="8"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="8">
         <v>21</v>
       </c>
@@ -2527,7 +2521,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="8">
         <v>22</v>
       </c>
@@ -2552,7 +2546,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="8">
         <v>23</v>
       </c>
@@ -2575,7 +2569,7 @@
       <c r="J24" s="8"/>
       <c r="K24" s="8"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="8">
         <v>24</v>
       </c>
@@ -2598,7 +2592,7 @@
       </c>
       <c r="K25" s="8"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="8">
         <v>25</v>
       </c>
@@ -2621,7 +2615,7 @@
       <c r="J26" s="8"/>
       <c r="K26" s="8"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="8">
         <v>26</v>
       </c>
@@ -2644,7 +2638,7 @@
       </c>
       <c r="K27" s="8"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="8">
         <v>27</v>
       </c>
@@ -2667,7 +2661,7 @@
       </c>
       <c r="K28" s="8"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="8">
         <v>28</v>
       </c>
@@ -2690,7 +2684,7 @@
       </c>
       <c r="K29" s="8"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="8">
         <v>29</v>
       </c>
@@ -2715,7 +2709,7 @@
       </c>
       <c r="K30" s="8"/>
     </row>
-    <row r="31" spans="1:11" ht="16.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8">
         <v>30</v>
       </c>
@@ -2738,7 +2732,7 @@
       </c>
       <c r="K31" s="8"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="8">
         <v>31</v>
       </c>
@@ -2763,7 +2757,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="8">
         <v>32</v>
       </c>
@@ -2788,7 +2782,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="8">
         <v>33</v>
       </c>
@@ -2811,7 +2805,7 @@
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="8">
         <v>34</v>
       </c>
@@ -2834,7 +2828,7 @@
       </c>
       <c r="K35" s="8"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="8">
         <v>35</v>
       </c>
@@ -2857,7 +2851,7 @@
       <c r="J36" s="8"/>
       <c r="K36" s="8"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="8">
         <v>36</v>
       </c>
@@ -2880,7 +2874,7 @@
       <c r="J37" s="8"/>
       <c r="K37" s="8"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="8">
         <v>37</v>
       </c>
@@ -2903,7 +2897,7 @@
       </c>
       <c r="K38" s="8"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="8">
         <v>38</v>
       </c>
@@ -2926,7 +2920,7 @@
       <c r="J39" s="8"/>
       <c r="K39" s="8"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="8">
         <v>39</v>
       </c>
@@ -2951,7 +2945,7 @@
       </c>
       <c r="K40" s="8"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="8">
         <v>40</v>
       </c>
@@ -2974,7 +2968,7 @@
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="8">
         <v>41</v>
       </c>
@@ -2997,7 +2991,7 @@
       <c r="J42" s="8"/>
       <c r="K42" s="8"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="8">
         <v>42</v>
       </c>
@@ -3022,7 +3016,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="8">
         <v>43</v>
       </c>
@@ -3045,7 +3039,7 @@
       <c r="J44" s="8"/>
       <c r="K44" s="8"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="8">
         <v>44</v>
       </c>
@@ -3070,7 +3064,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="8">
         <v>45</v>
       </c>
@@ -3095,7 +3089,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="8">
         <v>46</v>
       </c>
@@ -3120,7 +3114,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="8">
         <v>47</v>
       </c>
@@ -3145,7 +3139,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="8">
         <v>48</v>
       </c>
@@ -3166,7 +3160,7 @@
       </c>
       <c r="K49" s="8"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="8">
         <v>49</v>
       </c>
@@ -3191,7 +3185,7 @@
       </c>
       <c r="K50" s="8"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="8">
         <v>50</v>
       </c>
@@ -3216,7 +3210,7 @@
       </c>
       <c r="K51" s="8"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="8">
         <v>51</v>
       </c>
@@ -3241,7 +3235,7 @@
       </c>
       <c r="K52" s="8"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="8">
         <v>52</v>
       </c>
@@ -3264,7 +3258,7 @@
       <c r="J53" s="8"/>
       <c r="K53" s="8"/>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="8">
         <v>53</v>
       </c>
@@ -3289,7 +3283,7 @@
       </c>
       <c r="K54" s="8"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="8">
         <v>54</v>
       </c>
@@ -3312,7 +3306,7 @@
       <c r="J55" s="8"/>
       <c r="K55" s="8"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="8">
         <v>55</v>
       </c>
@@ -3335,7 +3329,7 @@
       <c r="J56" s="8"/>
       <c r="K56" s="8"/>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="8">
         <v>56</v>
       </c>
@@ -3358,7 +3352,7 @@
       <c r="J57" s="8"/>
       <c r="K57" s="8"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="8">
         <v>57</v>
       </c>
@@ -3381,7 +3375,7 @@
       </c>
       <c r="K58" s="8"/>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="8">
         <v>58</v>
       </c>
@@ -3402,7 +3396,7 @@
       </c>
       <c r="K59" s="8"/>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="8">
         <v>59</v>
       </c>
@@ -3427,7 +3421,7 @@
       </c>
       <c r="K60" s="8"/>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="8">
         <v>60</v>
       </c>
@@ -3450,7 +3444,7 @@
       </c>
       <c r="K61" s="8"/>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="8">
         <v>61</v>
       </c>
@@ -3473,7 +3467,7 @@
       <c r="J62" s="8"/>
       <c r="K62" s="8"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="8">
         <v>62</v>
       </c>
@@ -3494,7 +3488,7 @@
       <c r="J63" s="8"/>
       <c r="K63" s="8"/>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="8">
         <v>63</v>
       </c>
@@ -3517,7 +3511,7 @@
       <c r="J64" s="12"/>
       <c r="K64" s="8"/>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="8">
         <v>64</v>
       </c>
@@ -3538,7 +3532,7 @@
       <c r="J65" s="8"/>
       <c r="K65" s="8"/>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="8">
         <v>65</v>
       </c>
@@ -3561,7 +3555,7 @@
       <c r="J66" s="8"/>
       <c r="K66" s="8"/>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="8">
         <v>66</v>
       </c>
@@ -3582,7 +3576,7 @@
       </c>
       <c r="K67" s="8"/>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="8">
         <v>67</v>
       </c>
@@ -3609,7 +3603,7 @@
       </c>
       <c r="K68" s="8"/>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="8">
         <v>68</v>
       </c>
@@ -3630,7 +3624,7 @@
       <c r="J69" s="8"/>
       <c r="K69" s="8"/>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="8">
         <v>69</v>
       </c>
@@ -3653,7 +3647,7 @@
       <c r="J70" s="12"/>
       <c r="K70" s="8"/>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="8">
         <v>70</v>
       </c>
@@ -3676,7 +3670,7 @@
       <c r="J71" s="12"/>
       <c r="K71" s="8"/>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="8">
         <v>71</v>
       </c>
@@ -3699,7 +3693,7 @@
       </c>
       <c r="K72" s="8"/>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="8">
         <v>72</v>
       </c>
@@ -3728,7 +3722,7 @@
       </c>
       <c r="K73" s="8"/>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="8">
         <v>73</v>
       </c>
@@ -3753,7 +3747,7 @@
       <c r="J74" s="12"/>
       <c r="K74" s="8"/>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="8">
         <v>74</v>
       </c>
@@ -3776,7 +3770,7 @@
       <c r="J75" s="12"/>
       <c r="K75" s="8"/>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="8">
         <v>75</v>
       </c>
@@ -3799,7 +3793,7 @@
       </c>
       <c r="K76" s="8"/>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="8">
         <v>76</v>
       </c>
@@ -3822,7 +3816,7 @@
       <c r="J77" s="12"/>
       <c r="K77" s="8"/>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="8">
         <v>77</v>
       </c>
@@ -3845,7 +3839,7 @@
       </c>
       <c r="K78" s="8"/>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="8">
         <v>78</v>
       </c>
@@ -3868,7 +3862,7 @@
       </c>
       <c r="K79" s="8"/>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="8">
         <v>79</v>
       </c>
@@ -3891,7 +3885,7 @@
       <c r="J80" s="8"/>
       <c r="K80" s="8"/>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="8">
         <v>80</v>
       </c>
@@ -3912,7 +3906,7 @@
       <c r="J81" s="8"/>
       <c r="K81" s="8"/>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="8">
         <v>81</v>
       </c>
@@ -3935,7 +3929,7 @@
       <c r="J82" s="8"/>
       <c r="K82" s="8"/>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="8">
         <v>82</v>
       </c>
@@ -3956,7 +3950,7 @@
       <c r="J83" s="8"/>
       <c r="K83" s="8"/>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="8">
         <v>83</v>
       </c>
@@ -3976,12 +3970,14 @@
       <c r="G84" s="8"/>
       <c r="H84" s="8"/>
       <c r="I84" s="8"/>
-      <c r="J84" s="8"/>
+      <c r="J84" s="8" t="s">
+        <v>396</v>
+      </c>
       <c r="K84" s="8" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" s="8">
         <v>84</v>
       </c>
@@ -3996,17 +3992,19 @@
       </c>
       <c r="E85" s="8"/>
       <c r="F85" s="8" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="G85" s="8"/>
       <c r="H85" s="8"/>
       <c r="I85" s="8"/>
-      <c r="J85" s="8"/>
+      <c r="J85" s="8" t="s">
+        <v>391</v>
+      </c>
       <c r="K85" s="8" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="8">
         <v>85</v>
       </c>
@@ -4026,12 +4024,14 @@
       <c r="G86" s="8"/>
       <c r="H86" s="8"/>
       <c r="I86" s="8"/>
-      <c r="J86" s="8"/>
+      <c r="J86" s="8" t="s">
+        <v>214</v>
+      </c>
       <c r="K86" s="8" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" s="8">
         <v>86</v>
       </c>
@@ -4054,7 +4054,7 @@
       <c r="J87" s="8"/>
       <c r="K87" s="8"/>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" s="8">
         <v>87</v>
       </c>
@@ -4077,7 +4077,7 @@
       <c r="J88" s="8"/>
       <c r="K88" s="8"/>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" s="8">
         <v>88</v>
       </c>
@@ -4098,18 +4098,18 @@
       <c r="J89" s="8"/>
       <c r="K89" s="8"/>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" s="8">
         <v>89</v>
       </c>
       <c r="B90" s="8" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C90" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D90" s="16" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E90" s="8"/>
       <c r="F90" s="8" t="s">
@@ -4122,23 +4122,25 @@
         <v>113</v>
       </c>
       <c r="I90" s="8"/>
-      <c r="J90" s="8"/>
+      <c r="J90" s="8" t="s">
+        <v>391</v>
+      </c>
       <c r="K90" s="8" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" s="8">
         <v>90</v>
       </c>
       <c r="B91" s="8" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C91" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D91" s="16" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E91" s="8"/>
       <c r="F91" s="8" t="s">
@@ -4151,23 +4153,25 @@
         <v>113</v>
       </c>
       <c r="I91" s="8"/>
-      <c r="J91" s="8"/>
+      <c r="J91" s="8" t="s">
+        <v>396</v>
+      </c>
       <c r="K91" s="8" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" s="8">
         <v>91</v>
       </c>
       <c r="B92" s="8" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C92" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D92" s="16" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E92" s="8"/>
       <c r="F92" s="8" t="s">
@@ -4180,12 +4184,14 @@
         <v>113</v>
       </c>
       <c r="I92" s="8"/>
-      <c r="J92" s="8"/>
+      <c r="J92" s="8" t="s">
+        <v>214</v>
+      </c>
       <c r="K92" s="8" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" s="8">
         <v>92</v>
       </c>
@@ -4206,7 +4212,7 @@
       </c>
       <c r="K93" s="8"/>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" s="8">
         <v>93</v>
       </c>
@@ -4227,7 +4233,7 @@
       <c r="J94" s="8"/>
       <c r="K94" s="8"/>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95" s="8">
         <v>94</v>
       </c>
@@ -4250,7 +4256,7 @@
       <c r="J95" s="8"/>
       <c r="K95" s="8"/>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96" s="8">
         <v>95</v>
       </c>
@@ -4258,7 +4264,7 @@
         <v>174</v>
       </c>
       <c r="C96" s="8" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D96" s="8"/>
       <c r="E96" s="8"/>
@@ -4271,7 +4277,7 @@
       <c r="J96" s="8"/>
       <c r="K96" s="8"/>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A97" s="8">
         <v>96</v>
       </c>
@@ -4279,7 +4285,7 @@
         <v>175</v>
       </c>
       <c r="C97" s="8" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D97" s="8" t="s">
         <v>176</v>
@@ -4292,11 +4298,11 @@
       <c r="H97" s="8"/>
       <c r="I97" s="8"/>
       <c r="J97" s="8" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="K97" s="8"/>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A98" s="8">
         <v>97</v>
       </c>
@@ -4304,7 +4310,7 @@
         <v>178</v>
       </c>
       <c r="C98" s="8" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D98" s="8" t="s">
         <v>81</v>
@@ -4319,7 +4325,7 @@
       <c r="J98" s="8"/>
       <c r="K98" s="8"/>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A99" s="8">
         <v>98</v>
       </c>
@@ -4340,12 +4346,12 @@
       <c r="J99" s="8"/>
       <c r="K99" s="8"/>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A100" s="8">
         <v>99</v>
       </c>
       <c r="B100" s="8" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C100" s="8" t="s">
         <v>18</v>
@@ -4353,17 +4359,17 @@
       <c r="D100" s="8"/>
       <c r="E100" s="8"/>
       <c r="F100" s="8" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="G100" s="8"/>
       <c r="H100" s="8"/>
       <c r="I100" s="8"/>
       <c r="J100" s="8" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K100" s="8"/>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A101" s="8">
         <v>100</v>
       </c>
@@ -4374,7 +4380,7 @@
         <v>18</v>
       </c>
       <c r="D101" s="8" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="E101" s="8"/>
       <c r="F101" s="8" t="s">
@@ -4388,11 +4394,11 @@
       </c>
       <c r="I101" s="8"/>
       <c r="J101" s="8" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="K101" s="8"/>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A102" s="8">
         <v>101</v>
       </c>
@@ -4413,7 +4419,7 @@
       </c>
       <c r="K102" s="8"/>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A103" s="8">
         <v>102</v>
       </c>
@@ -4436,7 +4442,7 @@
       <c r="J103" s="8"/>
       <c r="K103" s="8"/>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A104" s="8">
         <v>103</v>
       </c>
@@ -4444,7 +4450,7 @@
         <v>184</v>
       </c>
       <c r="C104" s="8" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D104" s="8"/>
       <c r="E104" s="8"/>
@@ -4457,18 +4463,18 @@
       <c r="J104" s="8"/>
       <c r="K104" s="8"/>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A105" s="8">
         <v>104</v>
       </c>
       <c r="B105" s="8" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C105" s="8" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D105" s="8" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E105" s="8"/>
       <c r="F105" s="8" t="s">
@@ -4486,7 +4492,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A106" s="8">
         <v>105</v>
       </c>
@@ -4494,7 +4500,7 @@
         <v>185</v>
       </c>
       <c r="C106" s="8" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D106" s="8" t="s">
         <v>120</v>
@@ -4506,12 +4512,14 @@
       <c r="G106" s="8"/>
       <c r="H106" s="8"/>
       <c r="I106" s="8"/>
-      <c r="J106" s="8"/>
+      <c r="J106" s="8" t="s">
+        <v>400</v>
+      </c>
       <c r="K106" s="8" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A107" s="8">
         <v>106</v>
       </c>
@@ -4519,7 +4527,7 @@
         <v>187</v>
       </c>
       <c r="C107" s="8" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D107" s="8" t="s">
         <v>91</v>
@@ -4534,7 +4542,7 @@
       <c r="J107" s="8"/>
       <c r="K107" s="8"/>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A108" s="8">
         <v>107</v>
       </c>
@@ -4542,7 +4550,7 @@
         <v>188</v>
       </c>
       <c r="C108" s="8" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D108" s="8"/>
       <c r="E108" s="8"/>
@@ -4555,7 +4563,7 @@
       <c r="J108" s="8"/>
       <c r="K108" s="8"/>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A109" s="8">
         <v>108</v>
       </c>
@@ -4578,18 +4586,18 @@
       <c r="J109" s="8"/>
       <c r="K109" s="8"/>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A110" s="8">
         <v>109</v>
       </c>
       <c r="B110" s="8" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C110" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D110" s="16" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E110" s="8"/>
       <c r="F110" s="8" t="s">
@@ -4602,23 +4610,25 @@
         <v>113</v>
       </c>
       <c r="I110" s="8"/>
-      <c r="J110" s="8"/>
+      <c r="J110" s="8" t="s">
+        <v>391</v>
+      </c>
       <c r="K110" s="8" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A111" s="8">
         <v>110</v>
       </c>
       <c r="B111" s="8" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C111" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D111" s="16" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E111" s="8"/>
       <c r="F111" s="8" t="s">
@@ -4632,11 +4642,11 @@
       </c>
       <c r="I111" s="8"/>
       <c r="J111" s="8" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="K111" s="8"/>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A112" s="8">
         <v>111</v>
       </c>
@@ -4657,7 +4667,7 @@
       </c>
       <c r="K112" s="8"/>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113" s="8">
         <v>112</v>
       </c>
@@ -4678,7 +4688,7 @@
       <c r="J113" s="8"/>
       <c r="K113" s="8"/>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114" s="8">
         <v>113</v>
       </c>
@@ -4701,7 +4711,7 @@
       <c r="J114" s="8"/>
       <c r="K114" s="8"/>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" s="8">
         <v>114</v>
       </c>
@@ -4709,7 +4719,7 @@
         <v>193</v>
       </c>
       <c r="C115" s="8" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D115" s="8"/>
       <c r="E115" s="8"/>
@@ -4722,18 +4732,18 @@
       <c r="J115" s="8"/>
       <c r="K115" s="8"/>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" s="8">
         <v>115</v>
       </c>
       <c r="B116" s="8" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C116" s="8" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D116" s="8" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E116" s="8"/>
       <c r="F116" s="8" t="s">
@@ -4751,7 +4761,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" s="8">
         <v>116</v>
       </c>
@@ -4759,7 +4769,7 @@
         <v>194</v>
       </c>
       <c r="C117" s="8" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D117" s="8" t="s">
         <v>195</v>
@@ -4771,12 +4781,14 @@
       <c r="G117" s="8"/>
       <c r="H117" s="8"/>
       <c r="I117" s="8"/>
-      <c r="J117" s="8"/>
+      <c r="J117" s="8" t="s">
+        <v>408</v>
+      </c>
       <c r="K117" s="8" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" s="8">
         <v>117</v>
       </c>
@@ -4784,7 +4796,7 @@
         <v>197</v>
       </c>
       <c r="C118" s="8" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D118" s="8" t="s">
         <v>91</v>
@@ -4799,7 +4811,7 @@
       <c r="J118" s="8"/>
       <c r="K118" s="8"/>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" s="8">
         <v>118</v>
       </c>
@@ -4807,7 +4819,7 @@
         <v>198</v>
       </c>
       <c r="C119" s="8" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D119" s="8"/>
       <c r="E119" s="8"/>
@@ -4820,18 +4832,18 @@
       <c r="J119" s="8"/>
       <c r="K119" s="8"/>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" s="8">
         <v>119</v>
       </c>
       <c r="B120" s="8" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C120" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D120" s="16" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E120" s="8"/>
       <c r="F120" s="8" t="s">
@@ -4844,23 +4856,25 @@
         <v>113</v>
       </c>
       <c r="I120" s="8"/>
-      <c r="J120" s="8"/>
+      <c r="J120" s="8" t="s">
+        <v>391</v>
+      </c>
       <c r="K120" s="8" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" s="8">
         <v>120</v>
       </c>
       <c r="B121" s="8" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C121" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D121" s="16" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E121" s="8"/>
       <c r="F121" s="8" t="s">
@@ -4874,11 +4888,11 @@
       </c>
       <c r="I121" s="8"/>
       <c r="J121" s="8" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K121" s="8"/>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" s="8">
         <v>121</v>
       </c>
@@ -4899,7 +4913,7 @@
       </c>
       <c r="K122" s="8"/>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" s="8">
         <v>122</v>
       </c>
@@ -4922,7 +4936,7 @@
       <c r="J123" s="8"/>
       <c r="K123" s="8"/>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124" s="8">
         <v>123</v>
       </c>
@@ -4930,7 +4944,7 @@
         <v>202</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D124" s="8"/>
       <c r="E124" s="8"/>
@@ -4943,18 +4957,18 @@
       <c r="J124" s="8"/>
       <c r="K124" s="8"/>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125" s="8">
         <v>124</v>
       </c>
       <c r="B125" s="8" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C125" s="8" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D125" s="8" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E125" s="8"/>
       <c r="F125" s="8" t="s">
@@ -4972,7 +4986,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126" s="8">
         <v>125</v>
       </c>
@@ -4980,7 +4994,7 @@
         <v>203</v>
       </c>
       <c r="C126" s="8" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D126" s="8" t="s">
         <v>140</v>
@@ -4992,12 +5006,14 @@
       <c r="G126" s="8"/>
       <c r="H126" s="8"/>
       <c r="I126" s="8"/>
-      <c r="J126" s="8"/>
+      <c r="J126" s="8" t="s">
+        <v>409</v>
+      </c>
       <c r="K126" s="8" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127" s="8">
         <v>126</v>
       </c>
@@ -5005,7 +5021,7 @@
         <v>205</v>
       </c>
       <c r="C127" s="8" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D127" s="8" t="s">
         <v>143</v>
@@ -5020,7 +5036,7 @@
       <c r="J127" s="8"/>
       <c r="K127" s="8"/>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128" s="8">
         <v>127</v>
       </c>
@@ -5028,7 +5044,7 @@
         <v>206</v>
       </c>
       <c r="C128" s="8" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D128" s="8" t="s">
         <v>91</v>
@@ -5043,7 +5059,7 @@
       <c r="J128" s="8"/>
       <c r="K128" s="8"/>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A129" s="8">
         <v>128</v>
       </c>
@@ -5064,7 +5080,7 @@
       <c r="J129" s="8"/>
       <c r="K129" s="8"/>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A130" s="8">
         <v>129</v>
       </c>
@@ -5087,18 +5103,18 @@
       <c r="J130" s="8"/>
       <c r="K130" s="8"/>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A131" s="8">
         <v>130</v>
       </c>
       <c r="B131" s="8" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C131" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D131" s="16" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E131" s="8"/>
       <c r="F131" s="8" t="s">
@@ -5111,23 +5127,25 @@
         <v>113</v>
       </c>
       <c r="I131" s="8"/>
-      <c r="J131" s="8"/>
+      <c r="J131" s="8" t="s">
+        <v>391</v>
+      </c>
       <c r="K131" s="8" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A132" s="8">
         <v>131</v>
       </c>
       <c r="B132" s="8" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C132" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D132" s="16" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E132" s="8"/>
       <c r="F132" s="8" t="s">
@@ -5141,16 +5159,16 @@
       </c>
       <c r="I132" s="8"/>
       <c r="J132" s="8" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K132" s="8"/>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A133" s="8">
         <v>132</v>
       </c>
       <c r="B133" s="12" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C133" s="8" t="s">
         <v>18</v>
@@ -5166,7 +5184,7 @@
       <c r="J133" s="12"/>
       <c r="K133" s="8"/>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A134" s="8">
         <v>133</v>
       </c>
@@ -5189,7 +5207,7 @@
       <c r="J134" s="12"/>
       <c r="K134" s="8"/>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A135" s="8">
         <v>134</v>
       </c>
@@ -5212,7 +5230,7 @@
       </c>
       <c r="K135" s="8"/>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A136" s="8">
         <v>135</v>
       </c>
@@ -5235,7 +5253,7 @@
       <c r="J136" s="12"/>
       <c r="K136" s="8"/>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A137" s="8">
         <v>136</v>
       </c>
@@ -5243,7 +5261,7 @@
         <v>104</v>
       </c>
       <c r="C137" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D137" s="8" t="s">
         <v>105</v>
@@ -5255,12 +5273,14 @@
       <c r="G137" s="8"/>
       <c r="H137" s="8"/>
       <c r="I137" s="8"/>
-      <c r="J137" s="8"/>
+      <c r="J137" s="8" t="s">
+        <v>354</v>
+      </c>
       <c r="K137" s="8" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A138" s="8">
         <v>137</v>
       </c>
@@ -5268,7 +5288,7 @@
         <v>278</v>
       </c>
       <c r="C138" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D138" s="8"/>
       <c r="E138" s="8"/>
@@ -5283,7 +5303,7 @@
       </c>
       <c r="K138" s="8"/>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A139" s="8">
         <v>138</v>
       </c>
@@ -5291,7 +5311,7 @@
         <v>364</v>
       </c>
       <c r="C139" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D139" s="8" t="s">
         <v>108</v>
@@ -5306,7 +5326,7 @@
       <c r="J139" s="8"/>
       <c r="K139" s="8"/>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A140" s="8">
         <v>139</v>
       </c>
@@ -5314,7 +5334,7 @@
         <v>107</v>
       </c>
       <c r="C140" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D140" s="8" t="s">
         <v>365</v>
@@ -5333,7 +5353,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A141" s="8">
         <v>140</v>
       </c>
@@ -5341,7 +5361,7 @@
         <v>110</v>
       </c>
       <c r="C141" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D141" s="8" t="s">
         <v>111</v>
@@ -5353,12 +5373,14 @@
       <c r="G141" s="8"/>
       <c r="H141" s="8"/>
       <c r="I141" s="8"/>
-      <c r="J141" s="8"/>
+      <c r="J141" s="8" t="s">
+        <v>363</v>
+      </c>
       <c r="K141" s="8" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A142" s="8">
         <v>141</v>
       </c>
@@ -5366,7 +5388,7 @@
         <v>112</v>
       </c>
       <c r="C142" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D142" s="8" t="s">
         <v>81</v>
@@ -5381,7 +5403,7 @@
       <c r="J142" s="8"/>
       <c r="K142" s="8"/>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A143" s="8">
         <v>142</v>
       </c>
@@ -5400,18 +5422,18 @@
       <c r="J143" s="8"/>
       <c r="K143" s="8"/>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A144" s="8">
         <v>143</v>
       </c>
       <c r="B144" s="8" t="s">
-        <v>425</v>
+        <v>366</v>
       </c>
       <c r="C144" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D144" s="16" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E144" s="8"/>
       <c r="F144" s="8" t="s">
@@ -5429,18 +5451,18 @@
         <v>106</v>
       </c>
     </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A145" s="8">
         <v>144</v>
       </c>
       <c r="B145" s="8" t="s">
-        <v>424</v>
+        <v>366</v>
       </c>
       <c r="C145" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D145" s="16" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E145" s="8"/>
       <c r="F145" s="8" t="s">
@@ -5458,12 +5480,12 @@
         <v>109</v>
       </c>
     </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A146" s="8">
         <v>145</v>
       </c>
       <c r="B146" s="8" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C146" s="16"/>
       <c r="D146" s="16"/>
@@ -5479,7 +5501,7 @@
       </c>
       <c r="K146" s="8"/>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A147" s="8">
         <v>146</v>
       </c>
@@ -5502,7 +5524,7 @@
       <c r="J147" s="8"/>
       <c r="K147" s="8"/>
     </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A148" s="8">
         <v>147</v>
       </c>
@@ -5521,15 +5543,15 @@
       <c r="J148" s="8"/>
       <c r="K148" s="8"/>
     </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A149" s="8">
         <v>148</v>
       </c>
       <c r="B149" s="8" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C149" s="8" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D149" s="8" t="s">
         <v>164</v>
@@ -5541,20 +5563,22 @@
       <c r="G149" s="8"/>
       <c r="H149" s="8"/>
       <c r="I149" s="8"/>
-      <c r="J149" s="8"/>
+      <c r="J149" s="8" t="s">
+        <v>356</v>
+      </c>
       <c r="K149" s="8" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.35">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A150" s="8">
         <v>149</v>
       </c>
       <c r="B150" s="8" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C150" s="8" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D150" s="8" t="s">
         <v>81</v>
@@ -5569,7 +5593,7 @@
       <c r="J150" s="8"/>
       <c r="K150" s="8"/>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A151" s="8">
         <v>150</v>
       </c>
@@ -5588,18 +5612,18 @@
       <c r="J151" s="8"/>
       <c r="K151" s="8"/>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A152" s="8">
         <v>151</v>
       </c>
       <c r="B152" s="8" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C152" s="16" t="s">
         <v>18</v>
       </c>
       <c r="D152" s="16" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E152" s="8"/>
       <c r="F152" s="8" t="s">
@@ -5614,15 +5638,15 @@
       <c r="I152" s="8"/>
       <c r="J152" s="8"/>
       <c r="K152" s="8" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.35">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A153" s="8">
         <v>152</v>
       </c>
       <c r="B153" s="8" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C153" s="16"/>
       <c r="D153" s="16"/>
@@ -5638,12 +5662,12 @@
       </c>
       <c r="K153" s="8"/>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A154" s="8">
         <v>153</v>
       </c>
       <c r="B154" s="8" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C154" s="8" t="s">
         <v>18</v>
@@ -5661,18 +5685,18 @@
       <c r="J154" s="8"/>
       <c r="K154" s="8"/>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A155" s="8">
         <v>154</v>
       </c>
       <c r="B155" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C155" s="8" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D155" s="16" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E155" s="8"/>
       <c r="F155" s="8" t="s">
@@ -5690,18 +5714,18 @@
         <v>106</v>
       </c>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A156" s="8">
         <v>155</v>
       </c>
       <c r="B156" s="8" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C156" s="8" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D156" s="16" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E156" s="8"/>
       <c r="F156" s="8" t="s">
@@ -5719,15 +5743,15 @@
         <v>109</v>
       </c>
     </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A157" s="8">
         <v>156</v>
       </c>
       <c r="B157" s="8" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C157" s="8" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D157" s="16" t="s">
         <v>120</v>
@@ -5739,20 +5763,22 @@
       <c r="G157" s="8"/>
       <c r="H157" s="8"/>
       <c r="I157" s="8"/>
-      <c r="J157" s="8"/>
+      <c r="J157" s="8" t="s">
+        <v>357</v>
+      </c>
       <c r="K157" s="8" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A158" s="8">
         <v>157</v>
       </c>
       <c r="B158" s="8" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C158" s="8" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D158" s="8" t="s">
         <v>91</v>
@@ -5767,7 +5793,7 @@
       <c r="J158" s="8"/>
       <c r="K158" s="8"/>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A159" s="8">
         <v>158</v>
       </c>
@@ -5788,7 +5814,7 @@
       <c r="J159" s="8"/>
       <c r="K159" s="8"/>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A160" s="8">
         <v>159</v>
       </c>
@@ -5811,7 +5837,7 @@
       <c r="J160" s="8"/>
       <c r="K160" s="8"/>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A161" s="8">
         <v>160</v>
       </c>
@@ -5834,7 +5860,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A162" s="8">
         <v>161</v>
       </c>
@@ -5845,7 +5871,7 @@
         <v>18</v>
       </c>
       <c r="D162" s="8" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E162" s="8"/>
       <c r="F162" s="8" t="s">
@@ -5859,11 +5885,11 @@
       </c>
       <c r="I162" s="8"/>
       <c r="J162" s="8" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="K162" s="8"/>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A163" s="8">
         <v>162</v>
       </c>
@@ -5884,7 +5910,7 @@
       </c>
       <c r="K163" s="8"/>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A164" s="8">
         <v>163</v>
       </c>
@@ -5907,7 +5933,7 @@
       <c r="J164" s="8"/>
       <c r="K164" s="8"/>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A165" s="8">
         <v>164</v>
       </c>
@@ -5915,7 +5941,7 @@
         <v>128</v>
       </c>
       <c r="C165" s="8" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D165" s="8"/>
       <c r="E165" s="8"/>
@@ -5928,18 +5954,18 @@
       <c r="J165" s="8"/>
       <c r="K165" s="8"/>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A166" s="8">
         <v>165</v>
       </c>
       <c r="B166" s="8" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C166" s="8" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D166" s="16" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E166" s="8"/>
       <c r="F166" s="8" t="s">
@@ -5957,18 +5983,18 @@
         <v>106</v>
       </c>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A167" s="8">
         <v>166</v>
       </c>
       <c r="B167" s="8" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C167" s="8" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D167" s="16" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E167" s="8"/>
       <c r="F167" s="8" t="s">
@@ -5986,7 +6012,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A168" s="8">
         <v>167</v>
       </c>
@@ -5994,7 +6020,7 @@
         <v>129</v>
       </c>
       <c r="C168" s="8" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D168" s="8" t="s">
         <v>130</v>
@@ -6006,12 +6032,14 @@
       <c r="G168" s="8"/>
       <c r="H168" s="8"/>
       <c r="I168" s="8"/>
-      <c r="J168" s="8"/>
+      <c r="J168" s="8" t="s">
+        <v>358</v>
+      </c>
       <c r="K168" s="8" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A169" s="8">
         <v>168</v>
       </c>
@@ -6019,7 +6047,7 @@
         <v>132</v>
       </c>
       <c r="C169" s="8" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D169" s="8" t="s">
         <v>91</v>
@@ -6034,7 +6062,7 @@
       <c r="J169" s="8"/>
       <c r="K169" s="8"/>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A170" s="8">
         <v>169</v>
       </c>
@@ -6055,7 +6083,7 @@
       <c r="J170" s="8"/>
       <c r="K170" s="8"/>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A171" s="8">
         <v>170</v>
       </c>
@@ -6066,7 +6094,7 @@
         <v>18</v>
       </c>
       <c r="D171" s="8" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E171" s="8"/>
       <c r="F171" s="8" t="s">
@@ -6080,11 +6108,11 @@
       </c>
       <c r="I171" s="8"/>
       <c r="J171" s="8" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K171" s="8"/>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A172" s="8">
         <v>171</v>
       </c>
@@ -6105,7 +6133,7 @@
       </c>
       <c r="K172" s="8"/>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A173" s="8">
         <v>172</v>
       </c>
@@ -6128,7 +6156,7 @@
       <c r="J173" s="8"/>
       <c r="K173" s="8"/>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A174" s="8">
         <v>173</v>
       </c>
@@ -6136,7 +6164,7 @@
         <v>138</v>
       </c>
       <c r="C174" s="8" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D174" s="8"/>
       <c r="E174" s="8"/>
@@ -6149,18 +6177,18 @@
       <c r="J174" s="8"/>
       <c r="K174" s="8"/>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A175" s="8">
         <v>174</v>
       </c>
       <c r="B175" s="8" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C175" s="8" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D175" s="16" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E175" s="8"/>
       <c r="F175" s="8" t="s">
@@ -6178,18 +6206,18 @@
         <v>106</v>
       </c>
     </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A176" s="8">
         <v>175</v>
       </c>
       <c r="B176" s="8" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C176" s="8" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D176" s="16" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E176" s="8"/>
       <c r="F176" s="8" t="s">
@@ -6207,7 +6235,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A177" s="8">
         <v>176</v>
       </c>
@@ -6215,7 +6243,7 @@
         <v>139</v>
       </c>
       <c r="C177" s="8" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D177" s="8" t="s">
         <v>140</v>
@@ -6227,12 +6255,14 @@
       <c r="G177" s="8"/>
       <c r="H177" s="8"/>
       <c r="I177" s="8"/>
-      <c r="J177" s="8"/>
+      <c r="J177" s="8" t="s">
+        <v>359</v>
+      </c>
       <c r="K177" s="8" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A178" s="8">
         <v>177</v>
       </c>
@@ -6240,7 +6270,7 @@
         <v>142</v>
       </c>
       <c r="C178" s="8" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D178" s="8" t="s">
         <v>143</v>
@@ -6255,7 +6285,7 @@
       <c r="J178" s="8"/>
       <c r="K178" s="8"/>
     </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A179" s="8">
         <v>178</v>
       </c>
@@ -6263,7 +6293,7 @@
         <v>144</v>
       </c>
       <c r="C179" s="8" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D179" s="8" t="s">
         <v>91</v>
@@ -6278,7 +6308,7 @@
       <c r="J179" s="8"/>
       <c r="K179" s="8"/>
     </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A180" s="8">
         <v>179</v>
       </c>
@@ -6299,7 +6329,7 @@
       <c r="J180" s="8"/>
       <c r="K180" s="8"/>
     </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A181" s="8">
         <v>180</v>
       </c>
@@ -6322,7 +6352,7 @@
       <c r="J181" s="8"/>
       <c r="K181" s="8"/>
     </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A182" s="8">
         <v>181</v>
       </c>
@@ -6333,7 +6363,7 @@
         <v>18</v>
       </c>
       <c r="D182" s="8" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E182" s="8"/>
       <c r="F182" s="8" t="s">
@@ -6347,7 +6377,7 @@
       </c>
       <c r="I182" s="8"/>
       <c r="J182" s="8" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K182" s="8"/>
     </row>
@@ -6372,38 +6402,37 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31674DB1-2F1A-4DBC-BB88-9570360CDD29}">
-  <dimension ref="A1:AB2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AA2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="19.36328125" customWidth="1"/>
-    <col min="12" max="12" width="20.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.6328125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.6328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.6328125" customWidth="1"/>
-    <col min="19" max="19" width="22.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="23.6328125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="26.453125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.54296875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="23.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="22.36328125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="25" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="26.54296875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="19.28515625" customWidth="1"/>
+    <col min="12" max="12" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="25" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="29" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>45</v>
       </c>
@@ -6456,40 +6485,37 @@
         <v>118</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>426</v>
+        <v>121</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="AB1" s="1" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>210</v>
       </c>
@@ -6539,40 +6565,37 @@
         <v>355</v>
       </c>
       <c r="Q2" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
       <c r="R2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="S2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="T2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="U2" t="s">
-        <v>359</v>
+        <v>396</v>
       </c>
       <c r="V2" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="W2" t="s">
+        <v>214</v>
+      </c>
+      <c r="X2" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="X2" t="s">
-        <v>214</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>389</v>
+      <c r="Y2" t="s">
+        <v>400</v>
       </c>
       <c r="Z2" t="s">
-        <v>399</v>
+        <v>408</v>
       </c>
       <c r="AA2" t="s">
-        <v>407</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
   </sheetData>
@@ -6583,13 +6606,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A492E716-2E2C-4117-849D-EDDCA92E50F2}">
   <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.54296875" customWidth="1"/>
+    <col min="1" max="1" width="27.5703125" customWidth="1"/>
     <col min="2" max="2" width="95" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>215</v>
       </c>
@@ -6597,7 +6620,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>217</v>
       </c>
@@ -6605,7 +6628,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>219</v>
       </c>
@@ -6613,7 +6636,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>221</v>
       </c>
@@ -6621,7 +6644,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>223</v>
       </c>
@@ -6629,7 +6652,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>225</v>
       </c>
@@ -6637,7 +6660,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>227</v>
       </c>
@@ -6645,7 +6668,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>229</v>
       </c>
@@ -6653,7 +6676,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>231</v>
       </c>
@@ -6661,7 +6684,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>232</v>
       </c>
@@ -6669,7 +6692,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>233</v>
       </c>
@@ -6677,7 +6700,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>234</v>
       </c>
@@ -6685,7 +6708,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>236</v>
       </c>
@@ -6693,7 +6716,7 @@
         <v>46178</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>237</v>
       </c>
@@ -6701,7 +6724,7 @@
         <v>46178</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>238</v>
       </c>
@@ -6709,7 +6732,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>240</v>
       </c>
@@ -6717,7 +6740,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>242</v>
       </c>
@@ -6725,7 +6748,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>244</v>
       </c>
@@ -6733,7 +6756,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>245</v>
       </c>
@@ -6741,7 +6764,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>247</v>
       </c>
@@ -6757,14 +6780,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E342BCFB-0C06-449E-9D93-F79DC7BEEDFF}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="37" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>249</v>
       </c>
@@ -6775,7 +6798,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>38</v>
       </c>
@@ -6786,7 +6809,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -6797,7 +6820,7 @@
         <v>996289289229</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -6811,10 +6834,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{a4153a30-97aa-49dd-8839-66f72081522c}" enabled="1" method="Standard" siteId="{9ffff5c3-bdfa-4a9d-b595-ff68329945ef}" contentBits="0" removed="0"/>
-</clbl:labelList>
 </file>
</xml_diff>